<commit_message>
[SAE - Comunicaciones] Se agrega filtro para el usuario que tiene permiso 1707, listando todos los mensajes  creados por los usuarios. [SAI - Atenciones] Se corrige la validación del parámetro u,  evitando una repetición en el cargue de la página. Se agrega arreglo para el tipo de solución, manteniendo la opción "Se inicia caso" para las atenciones psicosociales y de terápias.
</commit_message>
<xml_diff>
--- a/Documentación/Estructura_DB_29_VISAE.xlsx
+++ b/Documentación/Estructura_DB_29_VISAE.xlsx
@@ -232,7 +232,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1447" uniqueCount="636">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1763" uniqueCount="791">
   <si>
     <t xml:space="preserve">App</t>
   </si>
@@ -2140,6 +2140,471 @@
   </si>
   <si>
     <t xml:space="preserve">visa45puntaje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa55sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa55idproyecto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sistemas VISAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visaesistemas.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plan04proyecto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plan04id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plan04numero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proyecto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa55codigo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Código</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa55id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa55nombre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa55descripcion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa55idresponsable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa55vigente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vigente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa55color</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa55fechacreacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa55fechaactualiza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha Actualización</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa56persemanal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa56consec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Periodos semanales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visaepersemanal.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa56id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa56agno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa56fechainicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha inicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa56fechafin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha fin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa56estado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 Abierto, 1 Cerrado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa56fechacreacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa56fechacierre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa56observacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57actividad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57idpersemanal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actividades VISAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visaeactividad.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57idsistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57consec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57titulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Titulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57descripcion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57tipoactividad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Programada, 2 Emergente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57estado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 Borrador, 1 Programada, 5 En proceso, 7 Ejecutada, 9 Reprogramada, 11 Cancelada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57prioridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Alta, 2 Media, 3 Baja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prioridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57fechaprogini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57fechaprogfin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57fechaejecini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57fechaejecfin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57porcentavance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57observacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57fechacreacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa57fechaactualiza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bsistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">btitulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bprioridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bfechaini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bfechafin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa58resultado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa58idactividad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resultados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visaeresultados.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa58consec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa58id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa58descripcion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa58cumplimiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 No cumplido, 1 Cumplido, 3 Parcial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumplimiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa58fecharegistro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha registro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa59evidencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa59idactividad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidencias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visaeevidencias.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa59consec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa59id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa59titulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Título</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa59idorigen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa59idarchivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa59tipoarchivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Documento, 3 Imagen, 5 Enlace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo de archivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa59descripcion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa59fechacarga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha cargue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa60reprograma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa60idactividad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reprogramación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visaereprograma.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa60consec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa60id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa60fechareproini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha inicial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa60fechareprofin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa60motivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa60fecharegistro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa61dificultad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa61idactividad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dificultades</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visaedificultad.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa61consec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa61id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa61descripcion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa61impacto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Alto, 2 Medio, 3 Bajo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impacto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa61requiereapoyo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requiere apoyo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa61fecharegistro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa62compromiso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa62idactividad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compromisos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visaecompromiso.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa62consec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa62id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa62descripcion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa62idresponsable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa62fechalimite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha límite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa62estado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pendiente, 2 En proceso, 3 Cumplido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa62fechacumple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa62observaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa62fecharegistro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa63solicitaapoyo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa63idactividad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solicitud de apoyo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visaesolicapoyo.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa63consec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa63id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa63descripcion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa63tipoapoyo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo de apoyo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa63idcolaborador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colaborador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa63estado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Pendiente, 2 En atención, 3 Resuelto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa63fechasolicitud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha solicitud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa63fecharespuesta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa63observaciones</t>
   </si>
 </sst>
 </file>
@@ -2149,7 +2614,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2174,7 +2639,7 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -2182,20 +2647,7 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -2311,7 +2763,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2324,23 +2776,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2364,23 +2816,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2388,7 +2840,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2412,11 +2864,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2425,10 +2877,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2548,14 +2996,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -2563,58 +3011,25 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
+          <a:miter/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
+          <a:miter/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
+          <a:miter/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -2632,48 +3047,12 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
@@ -8985,7 +9364,6 @@
       <c r="L316" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="T316" s="0"/>
       <c r="U316" s="1" t="n">
         <v>1</v>
       </c>
@@ -9003,7 +9381,6 @@
       <c r="L317" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="T317" s="0"/>
       <c r="U317" s="1" t="n">
         <v>2</v>
       </c>
@@ -9024,14 +9401,11 @@
       <c r="S318" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="T318" s="0"/>
       <c r="U318" s="1" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="319" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="T319" s="0"/>
-    </row>
+    <row r="319" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A320" s="1" t="s">
         <v>446</v>
@@ -9078,7 +9452,6 @@
       <c r="S320" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="T320" s="0"/>
       <c r="U320" s="1" t="n">
         <v>3</v>
       </c>
@@ -9099,7 +9472,6 @@
       <c r="L321" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="T321" s="0"/>
       <c r="U321" s="1" t="n">
         <v>1</v>
       </c>
@@ -9117,7 +9489,6 @@
       <c r="L322" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="T322" s="0"/>
       <c r="U322" s="1" t="n">
         <v>2</v>
       </c>
@@ -9138,7 +9509,6 @@
       <c r="S323" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="T323" s="0"/>
       <c r="U323" s="1" t="n">
         <v>4</v>
       </c>
@@ -9156,7 +9526,6 @@
       <c r="L324" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="T324" s="0"/>
       <c r="U324" s="1" t="n">
         <v>0</v>
       </c>
@@ -10790,7 +11159,7 @@
       <c r="G394" s="11"/>
       <c r="H394" s="11"/>
       <c r="I394" s="11"/>
-      <c r="J394" s="29"/>
+      <c r="J394" s="28"/>
       <c r="K394" s="11"/>
       <c r="L394" s="11"/>
       <c r="M394" s="11"/>
@@ -10821,7 +11190,7 @@
         <v>584</v>
       </c>
       <c r="I395" s="11"/>
-      <c r="J395" s="29"/>
+      <c r="J395" s="28"/>
       <c r="K395" s="11"/>
       <c r="L395" s="11"/>
       <c r="M395" s="11"/>
@@ -11499,7 +11868,2035 @@
         <v>3</v>
       </c>
     </row>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="429" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A429" s="1" t="s">
+        <v>636</v>
+      </c>
+      <c r="B429" s="1" t="s">
+        <v>637</v>
+      </c>
+      <c r="C429" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E429" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F429" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="G429" s="1" t="n">
+        <v>2955</v>
+      </c>
+      <c r="H429" s="1" t="s">
+        <v>638</v>
+      </c>
+      <c r="I429" s="1" t="s">
+        <v>639</v>
+      </c>
+      <c r="J429" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K429" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L429" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="N429" s="1" t="s">
+        <v>640</v>
+      </c>
+      <c r="O429" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="P429" s="1" t="s">
+        <v>642</v>
+      </c>
+      <c r="S429" s="1" t="s">
+        <v>643</v>
+      </c>
+      <c r="U429" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="430" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B430" s="1" t="s">
+        <v>644</v>
+      </c>
+      <c r="C430" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D430" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="E430" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K430" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="S430" s="1" t="s">
+        <v>645</v>
+      </c>
+      <c r="U430" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="431" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B431" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="C431" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K431" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L431" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U431" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="432" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B432" s="1" t="s">
+        <v>647</v>
+      </c>
+      <c r="C432" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D432" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="K432" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="U432" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="433" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B433" s="1" t="s">
+        <v>648</v>
+      </c>
+      <c r="C433" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D433" s="1" t="n">
+        <v>255</v>
+      </c>
+      <c r="K433" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="U433" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="434" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B434" s="1" t="s">
+        <v>649</v>
+      </c>
+      <c r="C434" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K434" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="L434" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="S434" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="U434" s="1" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="435" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B435" s="1" t="s">
+        <v>651</v>
+      </c>
+      <c r="C435" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K435" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="S435" s="1" t="s">
+        <v>652</v>
+      </c>
+      <c r="U435" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="436" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B436" s="1" t="s">
+        <v>653</v>
+      </c>
+      <c r="C436" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D436" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="K436" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="U436" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="437" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B437" s="1" t="s">
+        <v>654</v>
+      </c>
+      <c r="C437" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K437" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="L437" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="U437" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="438" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B438" s="1" t="s">
+        <v>655</v>
+      </c>
+      <c r="C438" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K438" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="L438" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="S438" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="U438" s="1" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="440" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A440" s="1" t="s">
+        <v>657</v>
+      </c>
+      <c r="B440" s="1" t="s">
+        <v>658</v>
+      </c>
+      <c r="C440" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E440" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F440" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="G440" s="1" t="n">
+        <v>2956</v>
+      </c>
+      <c r="H440" s="1" t="s">
+        <v>659</v>
+      </c>
+      <c r="I440" s="1" t="s">
+        <v>660</v>
+      </c>
+      <c r="J440" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K440" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L440" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U440" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="441" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B441" s="1" t="s">
+        <v>661</v>
+      </c>
+      <c r="C441" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K441" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L441" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U441" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="442" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B442" s="1" t="s">
+        <v>662</v>
+      </c>
+      <c r="C442" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K442" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="S442" s="1" t="s">
+        <v>663</v>
+      </c>
+      <c r="U442" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="443" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B443" s="1" t="s">
+        <v>664</v>
+      </c>
+      <c r="C443" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K443" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="L443" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="S443" s="1" t="s">
+        <v>665</v>
+      </c>
+      <c r="U443" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="444" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B444" s="1" t="s">
+        <v>666</v>
+      </c>
+      <c r="C444" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K444" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="L444" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="S444" s="1" t="s">
+        <v>667</v>
+      </c>
+      <c r="U444" s="1" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="445" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B445" s="1" t="s">
+        <v>668</v>
+      </c>
+      <c r="C445" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H445" s="1" t="s">
+        <v>669</v>
+      </c>
+      <c r="K445" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="L445" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="S445" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="U445" s="1" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="446" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B446" s="1" t="s">
+        <v>670</v>
+      </c>
+      <c r="C446" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K446" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="L446" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="U446" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="447" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B447" s="1" t="s">
+        <v>671</v>
+      </c>
+      <c r="C447" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K447" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L447" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="S447" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="U447" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="448" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B448" s="1" t="s">
+        <v>672</v>
+      </c>
+      <c r="C448" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D448" s="1" t="n">
+        <v>255</v>
+      </c>
+      <c r="K448" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="U448" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="450" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A450" s="1" t="s">
+        <v>673</v>
+      </c>
+      <c r="B450" s="1" t="s">
+        <v>674</v>
+      </c>
+      <c r="C450" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E450" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F450" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="G450" s="1" t="n">
+        <v>2957</v>
+      </c>
+      <c r="H450" s="1" t="s">
+        <v>675</v>
+      </c>
+      <c r="I450" s="1" t="s">
+        <v>676</v>
+      </c>
+      <c r="J450" s="1" t="n">
+        <v>2909</v>
+      </c>
+      <c r="K450" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L450" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="N450" s="1" t="n">
+        <v>2956</v>
+      </c>
+      <c r="O450" s="1" t="s">
+        <v>661</v>
+      </c>
+      <c r="U450" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="451" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B451" s="1" t="s">
+        <v>677</v>
+      </c>
+      <c r="C451" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E451" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K451" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L451" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="N451" s="1" t="s">
+        <v>636</v>
+      </c>
+      <c r="O451" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="P451" s="1" t="s">
+        <v>647</v>
+      </c>
+      <c r="S451" s="1" t="s">
+        <v>678</v>
+      </c>
+      <c r="U451" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="452" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B452" s="1" t="s">
+        <v>679</v>
+      </c>
+      <c r="C452" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E452" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K452" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L452" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U452" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="453" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B453" s="1" t="s">
+        <v>680</v>
+      </c>
+      <c r="C453" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K453" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="L453" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U453" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="454" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B454" s="1" t="s">
+        <v>681</v>
+      </c>
+      <c r="C454" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D454" s="1" t="n">
+        <v>200</v>
+      </c>
+      <c r="K454" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="S454" s="1" t="s">
+        <v>682</v>
+      </c>
+      <c r="U454" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="455" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B455" s="1" t="s">
+        <v>683</v>
+      </c>
+      <c r="C455" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K455" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U455" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="456" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B456" s="1" t="s">
+        <v>684</v>
+      </c>
+      <c r="C456" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H456" s="1" t="s">
+        <v>685</v>
+      </c>
+      <c r="K456" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="L456" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="U456" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="457" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B457" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="C457" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H457" s="1" t="s">
+        <v>687</v>
+      </c>
+      <c r="K457" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L457" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="M457" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="N457" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="O457" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="P457" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="Q457" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="S457" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="U457" s="1" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="458" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B458" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="C458" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H458" s="1" t="s">
+        <v>689</v>
+      </c>
+      <c r="K458" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="L458" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="S458" s="1" t="s">
+        <v>690</v>
+      </c>
+      <c r="U458" s="1" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="459" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B459" s="1" t="s">
+        <v>691</v>
+      </c>
+      <c r="C459" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K459" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="L459" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="S459" s="1" t="s">
+        <v>665</v>
+      </c>
+      <c r="U459" s="1" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="460" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B460" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C460" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K460" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="L460" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="S460" s="1" t="s">
+        <v>667</v>
+      </c>
+      <c r="U460" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="461" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B461" s="1" t="s">
+        <v>693</v>
+      </c>
+      <c r="C461" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K461" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="L461" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="U461" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="462" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B462" s="1" t="s">
+        <v>694</v>
+      </c>
+      <c r="C462" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K462" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="L462" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="U462" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="463" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B463" s="1" t="s">
+        <v>695</v>
+      </c>
+      <c r="C463" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K463" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="S463" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="U463" s="1" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="464" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B464" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="C464" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K464" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="U464" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="465" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B465" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C465" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K465" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="L465" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="U465" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="466" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B466" s="1" t="s">
+        <v>699</v>
+      </c>
+      <c r="C466" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K466" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="L466" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="U466" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="467" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B467" s="1" t="s">
+        <v>700</v>
+      </c>
+      <c r="C467" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K467" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="L467" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="N467" s="1" t="s">
+        <v>636</v>
+      </c>
+      <c r="O467" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="P467" s="1" t="s">
+        <v>644</v>
+      </c>
+      <c r="S467" s="1" t="s">
+        <v>678</v>
+      </c>
+      <c r="T467" s="1" t="s">
+        <v>677</v>
+      </c>
+      <c r="U467" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="468" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B468" s="1" t="s">
+        <v>701</v>
+      </c>
+      <c r="C468" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D468" s="1" t="n">
+        <v>200</v>
+      </c>
+      <c r="K468" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="L468" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="S468" s="1" t="s">
+        <v>682</v>
+      </c>
+      <c r="T468" s="1" t="s">
+        <v>681</v>
+      </c>
+      <c r="U468" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="469" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B469" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="C469" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K469" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="L469" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="N469" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="O469" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="P469" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="Q469" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="S469" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="T469" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="U469" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="470" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B470" s="1" t="s">
+        <v>702</v>
+      </c>
+      <c r="C470" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K470" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="L470" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="S470" s="1" t="s">
+        <v>690</v>
+      </c>
+      <c r="T470" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="U470" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="471" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B471" s="1" t="s">
+        <v>703</v>
+      </c>
+      <c r="C471" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K471" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="L471" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="S471" s="1" t="s">
+        <v>665</v>
+      </c>
+      <c r="T471" s="1" t="s">
+        <v>691</v>
+      </c>
+      <c r="U471" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="472" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B472" s="1" t="s">
+        <v>704</v>
+      </c>
+      <c r="C472" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K472" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="L472" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="S472" s="1" t="s">
+        <v>667</v>
+      </c>
+      <c r="T472" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="U472" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="474" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A474" s="1" t="s">
+        <v>705</v>
+      </c>
+      <c r="B474" s="9" t="s">
+        <v>706</v>
+      </c>
+      <c r="C474" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E474" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F474" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="G474" s="1" t="n">
+        <v>2958</v>
+      </c>
+      <c r="H474" s="1" t="s">
+        <v>707</v>
+      </c>
+      <c r="I474" s="1" t="s">
+        <v>708</v>
+      </c>
+      <c r="J474" s="1" t="n">
+        <v>2909</v>
+      </c>
+      <c r="K474" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L474" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="N474" s="1" t="n">
+        <v>2957</v>
+      </c>
+      <c r="O474" s="1" t="s">
+        <v>680</v>
+      </c>
+      <c r="U474" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="475" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B475" s="9" t="s">
+        <v>709</v>
+      </c>
+      <c r="C475" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E475" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K475" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L475" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U475" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="476" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B476" s="9" t="s">
+        <v>710</v>
+      </c>
+      <c r="C476" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K476" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L476" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U476" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="477" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B477" s="9" t="s">
+        <v>711</v>
+      </c>
+      <c r="C477" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K477" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="U477" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="478" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B478" s="9" t="s">
+        <v>712</v>
+      </c>
+      <c r="C478" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H478" s="1" t="s">
+        <v>713</v>
+      </c>
+      <c r="K478" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="L478" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="S478" s="1" t="s">
+        <v>714</v>
+      </c>
+      <c r="U478" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="479" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B479" s="9" t="s">
+        <v>715</v>
+      </c>
+      <c r="C479" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K479" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="L479" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="S479" s="1" t="s">
+        <v>716</v>
+      </c>
+      <c r="U479" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="481" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A481" s="1" t="s">
+        <v>717</v>
+      </c>
+      <c r="B481" s="1" t="s">
+        <v>718</v>
+      </c>
+      <c r="C481" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E481" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F481" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="G481" s="1" t="n">
+        <v>2959</v>
+      </c>
+      <c r="H481" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="I481" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="J481" s="1" t="n">
+        <v>2909</v>
+      </c>
+      <c r="K481" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L481" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="N481" s="1" t="n">
+        <v>2957</v>
+      </c>
+      <c r="O481" s="1" t="s">
+        <v>680</v>
+      </c>
+      <c r="U481" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="482" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B482" s="1" t="s">
+        <v>721</v>
+      </c>
+      <c r="C482" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E482" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K482" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L482" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U482" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="483" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B483" s="1" t="s">
+        <v>722</v>
+      </c>
+      <c r="C483" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K483" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L483" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U483" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="484" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B484" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="C484" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D484" s="1" t="n">
+        <v>255</v>
+      </c>
+      <c r="K484" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="S484" s="1" t="s">
+        <v>724</v>
+      </c>
+      <c r="U484" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="485" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B485" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C485" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K485" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="L485" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="U485" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="486" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B486" s="1" t="s">
+        <v>726</v>
+      </c>
+      <c r="C486" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K486" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="L486" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="U486" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="487" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B487" s="1" t="s">
+        <v>727</v>
+      </c>
+      <c r="C487" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H487" s="1" t="s">
+        <v>728</v>
+      </c>
+      <c r="K487" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="L487" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="S487" s="1" t="s">
+        <v>729</v>
+      </c>
+      <c r="U487" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="488" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B488" s="1" t="s">
+        <v>730</v>
+      </c>
+      <c r="C488" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D488" s="1" t="n">
+        <v>255</v>
+      </c>
+      <c r="K488" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="U488" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="489" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B489" s="1" t="s">
+        <v>731</v>
+      </c>
+      <c r="C489" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K489" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="L489" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="S489" s="1" t="s">
+        <v>732</v>
+      </c>
+      <c r="U489" s="1" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="491" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A491" s="1" t="s">
+        <v>733</v>
+      </c>
+      <c r="B491" s="1" t="s">
+        <v>734</v>
+      </c>
+      <c r="C491" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E491" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F491" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="G491" s="1" t="n">
+        <v>2960</v>
+      </c>
+      <c r="H491" s="1" t="s">
+        <v>735</v>
+      </c>
+      <c r="I491" s="1" t="s">
+        <v>736</v>
+      </c>
+      <c r="J491" s="1" t="n">
+        <v>2909</v>
+      </c>
+      <c r="K491" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L491" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="N491" s="1" t="n">
+        <v>2957</v>
+      </c>
+      <c r="O491" s="1" t="s">
+        <v>680</v>
+      </c>
+      <c r="U491" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="492" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B492" s="1" t="s">
+        <v>737</v>
+      </c>
+      <c r="C492" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E492" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K492" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L492" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U492" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="493" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B493" s="1" t="s">
+        <v>738</v>
+      </c>
+      <c r="C493" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K493" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L493" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U493" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="494" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B494" s="1" t="s">
+        <v>739</v>
+      </c>
+      <c r="C494" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K494" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="L494" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="S494" s="1" t="s">
+        <v>740</v>
+      </c>
+      <c r="U494" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="495" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B495" s="1" t="s">
+        <v>741</v>
+      </c>
+      <c r="C495" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K495" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="L495" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="S495" s="1" t="s">
+        <v>742</v>
+      </c>
+      <c r="U495" s="1" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="496" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B496" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="C496" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K496" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="S496" s="1" t="s">
+        <v>744</v>
+      </c>
+      <c r="U496" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="497" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B497" s="1" t="s">
+        <v>745</v>
+      </c>
+      <c r="C497" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K497" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="L497" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="U497" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="499" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A499" s="1" t="s">
+        <v>746</v>
+      </c>
+      <c r="B499" s="1" t="s">
+        <v>747</v>
+      </c>
+      <c r="C499" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E499" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F499" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="G499" s="1" t="n">
+        <v>2961</v>
+      </c>
+      <c r="H499" s="1" t="s">
+        <v>748</v>
+      </c>
+      <c r="I499" s="1" t="s">
+        <v>749</v>
+      </c>
+      <c r="J499" s="1" t="n">
+        <v>2909</v>
+      </c>
+      <c r="K499" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L499" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="N499" s="1" t="n">
+        <v>2957</v>
+      </c>
+      <c r="O499" s="1" t="s">
+        <v>680</v>
+      </c>
+      <c r="U499" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="500" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B500" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C500" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E500" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K500" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L500" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U500" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="501" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B501" s="1" t="s">
+        <v>751</v>
+      </c>
+      <c r="C501" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K501" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L501" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U501" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="502" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B502" s="1" t="s">
+        <v>752</v>
+      </c>
+      <c r="C502" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K502" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="U502" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="503" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B503" s="1" t="s">
+        <v>753</v>
+      </c>
+      <c r="C503" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H503" s="1" t="s">
+        <v>754</v>
+      </c>
+      <c r="K503" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="L503" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="S503" s="1" t="s">
+        <v>755</v>
+      </c>
+      <c r="U503" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="504" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B504" s="1" t="s">
+        <v>756</v>
+      </c>
+      <c r="C504" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K504" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="L504" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="S504" s="1" t="s">
+        <v>757</v>
+      </c>
+      <c r="U504" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="505" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B505" s="1" t="s">
+        <v>758</v>
+      </c>
+      <c r="C505" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K505" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="L505" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="S505" s="1" t="s">
+        <v>716</v>
+      </c>
+      <c r="U505" s="1" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="507" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A507" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="B507" s="1" t="s">
+        <v>760</v>
+      </c>
+      <c r="C507" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E507" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F507" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="G507" s="1" t="n">
+        <v>2962</v>
+      </c>
+      <c r="H507" s="1" t="s">
+        <v>761</v>
+      </c>
+      <c r="I507" s="1" t="s">
+        <v>762</v>
+      </c>
+      <c r="J507" s="1" t="n">
+        <v>2909</v>
+      </c>
+      <c r="K507" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L507" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="N507" s="1" t="n">
+        <v>2957</v>
+      </c>
+      <c r="O507" s="1" t="s">
+        <v>680</v>
+      </c>
+      <c r="U507" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="508" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B508" s="1" t="s">
+        <v>763</v>
+      </c>
+      <c r="C508" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E508" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K508" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L508" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U508" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="509" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B509" s="1" t="s">
+        <v>764</v>
+      </c>
+      <c r="C509" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K509" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L509" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U509" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="510" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B510" s="1" t="s">
+        <v>765</v>
+      </c>
+      <c r="C510" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K510" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="S510" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="U510" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="511" customFormat="false" ht="15" hidden="true" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="512" customFormat="false" ht="15" hidden="true" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="513" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B513" s="1" t="s">
+        <v>766</v>
+      </c>
+      <c r="C513" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K513" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="L513" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="S513" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="U513" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="514" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B514" s="1" t="s">
+        <v>767</v>
+      </c>
+      <c r="C514" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K514" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="L514" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="S514" s="1" t="s">
+        <v>768</v>
+      </c>
+      <c r="U514" s="1" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="515" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B515" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="C515" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H515" s="1" t="s">
+        <v>770</v>
+      </c>
+      <c r="K515" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="L515" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="M515" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="N515" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="O515" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="P515" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="Q515" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="S515" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="U515" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="516" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B516" s="1" t="s">
+        <v>771</v>
+      </c>
+      <c r="C516" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K516" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L516" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="U516" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="517" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B517" s="1" t="s">
+        <v>772</v>
+      </c>
+      <c r="C517" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K517" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="U517" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="518" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B518" s="1" t="s">
+        <v>773</v>
+      </c>
+      <c r="C518" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K518" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="L518" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="U518" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="520" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A520" s="1" t="s">
+        <v>774</v>
+      </c>
+      <c r="B520" s="1" t="s">
+        <v>775</v>
+      </c>
+      <c r="C520" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E520" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F520" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="G520" s="1" t="n">
+        <v>2963</v>
+      </c>
+      <c r="H520" s="1" t="s">
+        <v>776</v>
+      </c>
+      <c r="I520" s="1" t="s">
+        <v>777</v>
+      </c>
+      <c r="J520" s="1" t="n">
+        <v>2909</v>
+      </c>
+      <c r="K520" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L520" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="N520" s="1" t="n">
+        <v>2957</v>
+      </c>
+      <c r="O520" s="1" t="s">
+        <v>680</v>
+      </c>
+      <c r="U520" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="521" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B521" s="1" t="s">
+        <v>778</v>
+      </c>
+      <c r="C521" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E521" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K521" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L521" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U521" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="522" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B522" s="1" t="s">
+        <v>779</v>
+      </c>
+      <c r="C522" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K522" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L522" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U522" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="523" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B523" s="1" t="s">
+        <v>780</v>
+      </c>
+      <c r="C523" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K523" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="U523" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="524" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B524" s="1" t="s">
+        <v>781</v>
+      </c>
+      <c r="C524" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D524" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="K524" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="S524" s="1" t="s">
+        <v>782</v>
+      </c>
+      <c r="U524" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="525" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B525" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="C525" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K525" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="L525" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="S525" s="1" t="s">
+        <v>784</v>
+      </c>
+      <c r="U525" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="526" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B526" s="1" t="s">
+        <v>785</v>
+      </c>
+      <c r="C526" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H526" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="K526" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="L526" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="M526" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="N526" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="O526" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="P526" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="Q526" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="S526" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="U526" s="1" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="527" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B527" s="1" t="s">
+        <v>787</v>
+      </c>
+      <c r="C527" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K527" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L527" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="S527" s="1" t="s">
+        <v>788</v>
+      </c>
+      <c r="U527" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="528" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B528" s="1" t="s">
+        <v>789</v>
+      </c>
+      <c r="C528" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K528" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="L528" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="U528" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="529" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B529" s="1" t="s">
+        <v>790</v>
+      </c>
+      <c r="C529" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K529" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="U529" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
[SAE - Sistemas VISAE] Se organiza el módulo con  cada uno de los campos de entrada y se agrega el input color y la validación del hexadecimal. [SAE - Periodo Semanal] Se organiza el módulo con  cada uno de los campos de entrada. [SAE - Gestión Semanal] Entrega 2026-10-07. Se organiza el módulo de Actividades con  cada uno de los campos de entrada y la relación y validaciones con tablas hijas Compromisos, Dificultades, Reprogramación, Requiere Apoyo, Resultados y Evidencias. Implementación del módulo de Tablero de Control con las visualizaciones de filtros, cajas de datos, gráficos estadísticos y tablas de ejecución, alertas, decisiones, logros y calendario semanal.
</commit_message>
<xml_diff>
--- a/Documentación/Estructura_DB_29_VISAE.xlsx
+++ b/Documentación/Estructura_DB_29_VISAE.xlsx
@@ -232,7 +232,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1763" uniqueCount="791">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1757" uniqueCount="783">
   <si>
     <t xml:space="preserve">App</t>
   </si>
@@ -2220,13 +2220,7 @@
     <t xml:space="preserve">visa56id</t>
   </si>
   <si>
-    <t xml:space="preserve">visa56agno</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Año</t>
-  </si>
-  <si>
-    <t xml:space="preserve">visa56fechainicio</t>
+    <t xml:space="preserve">visa56fechaini</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha inicio</t>
@@ -2241,10 +2235,10 @@
     <t xml:space="preserve">visa56estado</t>
   </si>
   <si>
-    <t xml:space="preserve">0 Abierto, 1 Cerrado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">visa56fechacreacion</t>
+    <t xml:space="preserve">0 Cerrado, 1 Abierto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visa56fechacrea</t>
   </si>
   <si>
     <t xml:space="preserve">visa56fechacierre</t>
@@ -2253,6 +2247,9 @@
     <t xml:space="preserve">visa56observacion</t>
   </si>
   <si>
+    <t xml:space="preserve">visa56activo</t>
+  </si>
+  <si>
     <t xml:space="preserve">visa57actividad</t>
   </si>
   <si>
@@ -2319,16 +2316,13 @@
     <t xml:space="preserve">visa57fechaejecfin</t>
   </si>
   <si>
-    <t xml:space="preserve">visa57porcentavance</t>
+    <t xml:space="preserve">visa57porcavance</t>
   </si>
   <si>
     <t xml:space="preserve">Avance</t>
   </si>
   <si>
-    <t xml:space="preserve">visa57observacion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">visa57fechacreacion</t>
+    <t xml:space="preserve">visa57fechacrea</t>
   </si>
   <si>
     <t xml:space="preserve">visa57fechaactualiza</t>
@@ -2358,9 +2352,6 @@
     <t xml:space="preserve">Resultados</t>
   </si>
   <si>
-    <t xml:space="preserve">visaeresultados.php</t>
-  </si>
-  <si>
     <t xml:space="preserve">visa58consec</t>
   </si>
   <si>
@@ -2373,7 +2364,7 @@
     <t xml:space="preserve">visa58cumplimiento</t>
   </si>
   <si>
-    <t xml:space="preserve">0 No cumplido, 1 Cumplido, 3 Parcial</t>
+    <t xml:space="preserve">1 No cumplido, 3 Cumplido, 5 Parcial</t>
   </si>
   <si>
     <t xml:space="preserve">Cumplimiento</t>
@@ -2394,9 +2385,6 @@
     <t xml:space="preserve">Evidencias</t>
   </si>
   <si>
-    <t xml:space="preserve">visaeevidencias.php</t>
-  </si>
-  <si>
     <t xml:space="preserve">visa59consec</t>
   </si>
   <si>
@@ -2433,6 +2421,9 @@
     <t xml:space="preserve">Fecha cargue</t>
   </si>
   <si>
+    <t xml:space="preserve">visa59idusuario</t>
+  </si>
+  <si>
     <t xml:space="preserve">visa60reprograma</t>
   </si>
   <si>
@@ -2442,9 +2433,6 @@
     <t xml:space="preserve">Reprogramación</t>
   </si>
   <si>
-    <t xml:space="preserve">visaereprograma.php</t>
-  </si>
-  <si>
     <t xml:space="preserve">visa60consec</t>
   </si>
   <si>
@@ -2472,6 +2460,9 @@
     <t xml:space="preserve">visa60fecharegistro</t>
   </si>
   <si>
+    <t xml:space="preserve">visa60idusuario</t>
+  </si>
+  <si>
     <t xml:space="preserve">visa61dificultad</t>
   </si>
   <si>
@@ -2481,9 +2472,6 @@
     <t xml:space="preserve">Dificultades</t>
   </si>
   <si>
-    <t xml:space="preserve">visaedificultad.php</t>
-  </si>
-  <si>
     <t xml:space="preserve">visa61consec</t>
   </si>
   <si>
@@ -2520,9 +2508,6 @@
     <t xml:space="preserve">Compromisos</t>
   </si>
   <si>
-    <t xml:space="preserve">visaecompromiso.php</t>
-  </si>
-  <si>
     <t xml:space="preserve">visa62consec</t>
   </si>
   <si>
@@ -2565,9 +2550,6 @@
     <t xml:space="preserve">Solicitud de apoyo</t>
   </si>
   <si>
-    <t xml:space="preserve">visaesolicapoyo.php</t>
-  </si>
-  <si>
     <t xml:space="preserve">visa63consec</t>
   </si>
   <si>
@@ -2575,12 +2557,6 @@
   </si>
   <si>
     <t xml:space="preserve">visa63descripcion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">visa63tipoapoyo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tipo de apoyo</t>
   </si>
   <si>
     <t xml:space="preserve">visa63idcolaborador</t>
@@ -11931,6 +11907,7 @@
       <c r="E430" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="J430" s="1"/>
       <c r="K430" s="1" t="n">
         <v>2</v>
       </c>
@@ -11948,6 +11925,7 @@
       <c r="C431" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J431" s="1"/>
       <c r="K431" s="1" t="n">
         <v>3</v>
       </c>
@@ -11968,6 +11946,7 @@
       <c r="D432" s="1" t="n">
         <v>100</v>
       </c>
+      <c r="J432" s="1"/>
       <c r="K432" s="1" t="n">
         <v>4</v>
       </c>
@@ -11980,11 +11959,9 @@
         <v>648</v>
       </c>
       <c r="C433" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D433" s="1" t="n">
-        <v>255</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="J433" s="1"/>
       <c r="K433" s="1" t="n">
         <v>5</v>
       </c>
@@ -11999,6 +11976,7 @@
       <c r="C434" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J434" s="1"/>
       <c r="K434" s="1" t="n">
         <v>6</v>
       </c>
@@ -12019,8 +11997,12 @@
       <c r="C435" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J435" s="1"/>
       <c r="K435" s="1" t="n">
         <v>7</v>
+      </c>
+      <c r="L435" s="1" t="n">
+        <v>3</v>
       </c>
       <c r="S435" s="1" t="s">
         <v>652</v>
@@ -12034,13 +12016,14 @@
         <v>653</v>
       </c>
       <c r="C436" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D436" s="1" t="n">
-        <v>16</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="J436" s="1"/>
       <c r="K436" s="1" t="n">
         <v>8</v>
+      </c>
+      <c r="L436" s="1" t="n">
+        <v>3</v>
       </c>
       <c r="U436" s="1" t="n">
         <v>0</v>
@@ -12053,11 +12036,15 @@
       <c r="C437" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J437" s="1"/>
       <c r="K437" s="1" t="n">
         <v>9</v>
       </c>
       <c r="L437" s="1" t="n">
         <v>7</v>
+      </c>
+      <c r="M437" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="U437" s="1" t="n">
         <v>0</v>
@@ -12070,18 +12057,25 @@
       <c r="C438" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J438" s="1"/>
       <c r="K438" s="1" t="n">
         <v>10</v>
       </c>
       <c r="L438" s="1" t="n">
         <v>7</v>
       </c>
+      <c r="M438" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="S438" s="1" t="s">
         <v>656</v>
       </c>
       <c r="U438" s="1" t="n">
         <v>6</v>
       </c>
+    </row>
+    <row r="439" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="J439" s="1"/>
     </row>
     <row r="440" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A440" s="1" t="s">
@@ -12128,6 +12122,7 @@
       <c r="C441" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J441" s="1"/>
       <c r="K441" s="1" t="n">
         <v>2</v>
       </c>
@@ -12145,14 +12140,18 @@
       <c r="C442" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J442" s="1"/>
       <c r="K442" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="L442" s="1" t="n">
+        <v>7</v>
       </c>
       <c r="S442" s="1" t="s">
         <v>663</v>
       </c>
       <c r="U442" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="443" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12162,6 +12161,7 @@
       <c r="C443" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J443" s="1"/>
       <c r="K443" s="1" t="n">
         <v>4</v>
       </c>
@@ -12172,7 +12172,7 @@
         <v>665</v>
       </c>
       <c r="U443" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="444" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12182,17 +12182,21 @@
       <c r="C444" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="H444" s="1" t="s">
+        <v>667</v>
+      </c>
+      <c r="J444" s="1"/>
       <c r="K444" s="1" t="n">
         <v>5</v>
       </c>
       <c r="L444" s="1" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="S444" s="1" t="s">
-        <v>667</v>
+        <v>502</v>
       </c>
       <c r="U444" s="1" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="445" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12202,82 +12206,77 @@
       <c r="C445" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H445" s="1" t="s">
-        <v>669</v>
-      </c>
+      <c r="J445" s="1"/>
       <c r="K445" s="1" t="n">
         <v>6</v>
       </c>
       <c r="L445" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="S445" s="1" t="s">
-        <v>502</v>
+        <v>7</v>
       </c>
       <c r="U445" s="1" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="446" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B446" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="C446" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J446" s="1"/>
       <c r="K446" s="1" t="n">
         <v>7</v>
       </c>
       <c r="L446" s="1" t="n">
         <v>7</v>
       </c>
+      <c r="S446" s="1" t="s">
+        <v>518</v>
+      </c>
       <c r="U446" s="1" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="447" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B447" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="C447" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="J447" s="1"/>
       <c r="K447" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="L447" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="S447" s="1" t="s">
-        <v>518</v>
-      </c>
       <c r="U447" s="1" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="448" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B448" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="C448" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D448" s="1" t="n">
-        <v>255</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="J448" s="1"/>
       <c r="K448" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="U448" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="L448" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="449" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="J449" s="1"/>
     </row>
     <row r="450" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A450" s="1" t="s">
+        <v>672</v>
+      </c>
+      <c r="B450" s="1" t="s">
         <v>673</v>
-      </c>
-      <c r="B450" s="1" t="s">
-        <v>674</v>
       </c>
       <c r="C450" s="1" t="s">
         <v>18</v>
@@ -12292,10 +12291,10 @@
         <v>2957</v>
       </c>
       <c r="H450" s="1" t="s">
+        <v>674</v>
+      </c>
+      <c r="I450" s="1" t="s">
         <v>675</v>
-      </c>
-      <c r="I450" s="1" t="s">
-        <v>676</v>
       </c>
       <c r="J450" s="1" t="n">
         <v>2909</v>
@@ -12304,21 +12303,24 @@
         <v>1</v>
       </c>
       <c r="L450" s="1" t="n">
-        <v>52</v>
-      </c>
-      <c r="N450" s="1" t="n">
-        <v>2956</v>
+        <v>3</v>
+      </c>
+      <c r="N450" s="1" t="s">
+        <v>657</v>
       </c>
       <c r="O450" s="1" t="s">
         <v>661</v>
       </c>
+      <c r="P450" s="1" t="s">
+        <v>662</v>
+      </c>
       <c r="U450" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="451" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B451" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="C451" s="1" t="s">
         <v>18</v>
@@ -12326,11 +12328,12 @@
       <c r="E451" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="J451" s="1"/>
       <c r="K451" s="1" t="n">
         <v>2</v>
       </c>
       <c r="L451" s="1" t="n">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="N451" s="1" t="s">
         <v>636</v>
@@ -12342,7 +12345,7 @@
         <v>647</v>
       </c>
       <c r="S451" s="1" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="U451" s="1" t="n">
         <v>2</v>
@@ -12350,7 +12353,7 @@
     </row>
     <row r="452" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B452" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="C452" s="1" t="s">
         <v>18</v>
@@ -12358,6 +12361,7 @@
       <c r="E452" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="J452" s="1"/>
       <c r="K452" s="1" t="n">
         <v>3</v>
       </c>
@@ -12370,11 +12374,12 @@
     </row>
     <row r="453" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B453" s="1" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="C453" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J453" s="1"/>
       <c r="K453" s="1" t="n">
         <v>4</v>
       </c>
@@ -12387,7 +12392,7 @@
     </row>
     <row r="454" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B454" s="1" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="C454" s="1" t="s">
         <v>30</v>
@@ -12395,11 +12400,12 @@
       <c r="D454" s="1" t="n">
         <v>200</v>
       </c>
+      <c r="J454" s="1"/>
       <c r="K454" s="1" t="n">
         <v>5</v>
       </c>
       <c r="S454" s="1" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="U454" s="1" t="n">
         <v>3</v>
@@ -12407,11 +12413,12 @@
     </row>
     <row r="455" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B455" s="1" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="C455" s="1" t="s">
         <v>113</v>
       </c>
+      <c r="J455" s="1"/>
       <c r="K455" s="1" t="n">
         <v>6</v>
       </c>
@@ -12421,14 +12428,15 @@
     </row>
     <row r="456" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B456" s="1" t="s">
+        <v>683</v>
+      </c>
+      <c r="C456" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H456" s="1" t="s">
         <v>684</v>
       </c>
-      <c r="C456" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H456" s="1" t="s">
-        <v>685</v>
-      </c>
+      <c r="J456" s="1"/>
       <c r="K456" s="1" t="n">
         <v>7</v>
       </c>
@@ -12441,22 +12449,23 @@
     </row>
     <row r="457" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B457" s="1" t="s">
+        <v>685</v>
+      </c>
+      <c r="C457" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H457" s="1" t="s">
         <v>686</v>
       </c>
-      <c r="C457" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H457" s="1" t="s">
-        <v>687</v>
-      </c>
+      <c r="J457" s="1"/>
       <c r="K457" s="1" t="n">
         <v>8</v>
       </c>
       <c r="L457" s="1" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="M457" s="1" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="N457" s="1" t="s">
         <v>498</v>
@@ -12479,14 +12488,15 @@
     </row>
     <row r="458" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B458" s="1" t="s">
+        <v>687</v>
+      </c>
+      <c r="C458" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H458" s="1" t="s">
         <v>688</v>
       </c>
-      <c r="C458" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H458" s="1" t="s">
-        <v>689</v>
-      </c>
+      <c r="J458" s="1"/>
       <c r="K458" s="1" t="n">
         <v>9</v>
       </c>
@@ -12494,7 +12504,7 @@
         <v>3</v>
       </c>
       <c r="S458" s="1" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="U458" s="1" t="n">
         <v>7</v>
@@ -12502,11 +12512,12 @@
     </row>
     <row r="459" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B459" s="1" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="C459" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J459" s="1"/>
       <c r="K459" s="1" t="n">
         <v>10</v>
       </c>
@@ -12514,7 +12525,7 @@
         <v>7</v>
       </c>
       <c r="S459" s="1" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="U459" s="1" t="n">
         <v>4</v>
@@ -12522,11 +12533,12 @@
     </row>
     <row r="460" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B460" s="1" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="C460" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J460" s="1"/>
       <c r="K460" s="1" t="n">
         <v>11</v>
       </c>
@@ -12534,7 +12546,7 @@
         <v>7</v>
       </c>
       <c r="S460" s="1" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="U460" s="1" t="n">
         <v>5</v>
@@ -12542,11 +12554,12 @@
     </row>
     <row r="461" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B461" s="1" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="C461" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J461" s="1"/>
       <c r="K461" s="1" t="n">
         <v>12</v>
       </c>
@@ -12559,11 +12572,12 @@
     </row>
     <row r="462" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B462" s="1" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="C462" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J462" s="1"/>
       <c r="K462" s="1" t="n">
         <v>13</v>
       </c>
@@ -12576,16 +12590,17 @@
     </row>
     <row r="463" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B463" s="1" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="C463" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>400</v>
+      </c>
+      <c r="J463" s="1"/>
       <c r="K463" s="1" t="n">
         <v>14</v>
       </c>
       <c r="S463" s="1" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="U463" s="1" t="n">
         <v>8</v>
@@ -12593,47 +12608,74 @@
     </row>
     <row r="464" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B464" s="1" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C464" s="1" t="s">
-        <v>113</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="J464" s="1"/>
       <c r="K464" s="1" t="n">
         <v>15</v>
       </c>
+      <c r="L464" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="M464" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="U464" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="465" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B465" s="1" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C465" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J465" s="1"/>
       <c r="K465" s="1" t="n">
         <v>16</v>
       </c>
       <c r="L465" s="1" t="n">
         <v>7</v>
       </c>
+      <c r="M465" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="U465" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="466" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B466" s="1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C466" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J466" s="1"/>
       <c r="K466" s="1" t="n">
         <v>17</v>
       </c>
       <c r="L466" s="1" t="n">
-        <v>7</v>
+        <v>23</v>
+      </c>
+      <c r="N466" s="1" t="s">
+        <v>636</v>
+      </c>
+      <c r="O466" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="P466" s="1" t="s">
+        <v>644</v>
+      </c>
+      <c r="S466" s="1" t="s">
+        <v>677</v>
+      </c>
+      <c r="T466" s="1" t="s">
+        <v>676</v>
       </c>
       <c r="U466" s="1" t="n">
         <v>0</v>
@@ -12641,31 +12683,26 @@
     </row>
     <row r="467" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B467" s="1" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="C467" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="D467" s="1" t="n">
+        <v>200</v>
+      </c>
+      <c r="J467" s="1"/>
       <c r="K467" s="1" t="n">
         <v>18</v>
       </c>
       <c r="L467" s="1" t="n">
-        <v>23</v>
-      </c>
-      <c r="N467" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="O467" s="1" t="s">
-        <v>646</v>
-      </c>
-      <c r="P467" s="1" t="s">
-        <v>644</v>
+        <v>22</v>
       </c>
       <c r="S467" s="1" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
       <c r="T467" s="1" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
       <c r="U467" s="1" t="n">
         <v>0</v>
@@ -12673,25 +12710,35 @@
     </row>
     <row r="468" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B468" s="1" t="s">
-        <v>701</v>
+        <v>534</v>
       </c>
       <c r="C468" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D468" s="1" t="n">
-        <v>200</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="J468" s="1"/>
       <c r="K468" s="1" t="n">
         <v>19</v>
       </c>
       <c r="L468" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="N468" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="O468" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="P468" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="Q468" s="1" t="s">
+        <v>501</v>
       </c>
       <c r="S468" s="1" t="s">
-        <v>682</v>
+        <v>502</v>
       </c>
       <c r="T468" s="1" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="U468" s="1" t="n">
         <v>0</v>
@@ -12699,34 +12746,23 @@
     </row>
     <row r="469" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B469" s="1" t="s">
-        <v>534</v>
+        <v>700</v>
       </c>
       <c r="C469" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J469" s="1"/>
       <c r="K469" s="1" t="n">
         <v>20</v>
       </c>
       <c r="L469" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="N469" s="1" t="s">
-        <v>498</v>
-      </c>
-      <c r="O469" s="1" t="s">
-        <v>499</v>
-      </c>
-      <c r="P469" s="1" t="s">
-        <v>500</v>
-      </c>
-      <c r="Q469" s="1" t="s">
-        <v>501</v>
-      </c>
       <c r="S469" s="1" t="s">
-        <v>502</v>
+        <v>689</v>
       </c>
       <c r="T469" s="1" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="U469" s="1" t="n">
         <v>0</v>
@@ -12734,22 +12770,23 @@
     </row>
     <row r="470" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B470" s="1" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C470" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J470" s="1"/>
       <c r="K470" s="1" t="n">
         <v>21</v>
       </c>
       <c r="L470" s="1" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="S470" s="1" t="s">
+        <v>663</v>
+      </c>
+      <c r="T470" s="1" t="s">
         <v>690</v>
-      </c>
-      <c r="T470" s="1" t="s">
-        <v>688</v>
       </c>
       <c r="U470" s="1" t="n">
         <v>0</v>
@@ -12757,11 +12794,12 @@
     </row>
     <row r="471" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B471" s="1" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C471" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J471" s="1"/>
       <c r="K471" s="1" t="n">
         <v>22</v>
       </c>
@@ -12779,33 +12817,49 @@
       </c>
     </row>
     <row r="472" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B472" s="1" t="s">
+      <c r="J472" s="1"/>
+    </row>
+    <row r="473" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A473" s="1" t="s">
+        <v>703</v>
+      </c>
+      <c r="B473" s="1" t="s">
         <v>704</v>
       </c>
-      <c r="C472" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K472" s="1" t="n">
-        <v>23</v>
-      </c>
-      <c r="L472" s="1" t="n">
-        <v>27</v>
-      </c>
-      <c r="S472" s="1" t="s">
-        <v>667</v>
-      </c>
-      <c r="T472" s="1" t="s">
-        <v>692</v>
-      </c>
-      <c r="U472" s="1" t="n">
+      <c r="C473" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E473" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F473" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="G473" s="1" t="n">
+        <v>2958</v>
+      </c>
+      <c r="H473" s="1" t="s">
+        <v>705</v>
+      </c>
+      <c r="J473" s="1"/>
+      <c r="K473" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L473" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="N473" s="1" t="n">
+        <v>2957</v>
+      </c>
+      <c r="O473" s="1" t="s">
+        <v>679</v>
+      </c>
+      <c r="U473" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="474" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A474" s="1" t="s">
-        <v>705</v>
-      </c>
-      <c r="B474" s="9" t="s">
+      <c r="B474" s="1" t="s">
         <v>706</v>
       </c>
       <c r="C474" s="1" t="s">
@@ -12814,137 +12868,143 @@
       <c r="E474" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F474" s="1" t="n">
-        <v>29</v>
-      </c>
-      <c r="G474" s="1" t="n">
-        <v>2958</v>
-      </c>
-      <c r="H474" s="1" t="s">
+      <c r="J474" s="1"/>
+      <c r="K474" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L474" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U474" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="475" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B475" s="1" t="s">
         <v>707</v>
       </c>
-      <c r="I474" s="1" t="s">
-        <v>708</v>
-      </c>
-      <c r="J474" s="1" t="n">
-        <v>2909</v>
-      </c>
-      <c r="K474" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="L474" s="1" t="n">
-        <v>52</v>
-      </c>
-      <c r="N474" s="1" t="n">
-        <v>2957</v>
-      </c>
-      <c r="O474" s="1" t="s">
-        <v>680</v>
-      </c>
-      <c r="U474" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="475" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B475" s="9" t="s">
-        <v>709</v>
-      </c>
       <c r="C475" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E475" s="1" t="s">
-        <v>19</v>
-      </c>
+      <c r="J475" s="1"/>
       <c r="K475" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L475" s="1" t="n">
         <v>6</v>
       </c>
       <c r="U475" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="476" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B476" s="9" t="s">
-        <v>710</v>
+      <c r="B476" s="1" t="s">
+        <v>708</v>
       </c>
       <c r="C476" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="J476" s="1"/>
       <c r="K476" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="L476" s="1" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U476" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="477" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B477" s="9" t="s">
+      <c r="B477" s="1" t="s">
+        <v>709</v>
+      </c>
+      <c r="C477" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H477" s="1" t="s">
+        <v>710</v>
+      </c>
+      <c r="J477" s="1"/>
+      <c r="K477" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="L477" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="S477" s="1" t="s">
         <v>711</v>
       </c>
-      <c r="C477" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="K477" s="1" t="n">
-        <v>4</v>
-      </c>
       <c r="U477" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="478" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B478" s="1" t="s">
+        <v>712</v>
+      </c>
+      <c r="C478" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J478" s="1"/>
+      <c r="K478" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="L478" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="M478" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="S478" s="1" t="s">
+        <v>713</v>
+      </c>
+      <c r="U478" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="479" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="J479" s="1"/>
+    </row>
+    <row r="480" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A480" s="1" t="s">
+        <v>714</v>
+      </c>
+      <c r="B480" s="1" t="s">
+        <v>715</v>
+      </c>
+      <c r="C480" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E480" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F480" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="G480" s="1" t="n">
+        <v>2959</v>
+      </c>
+      <c r="H480" s="1" t="s">
+        <v>716</v>
+      </c>
+      <c r="J480" s="1"/>
+      <c r="K480" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L480" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="N480" s="1" t="n">
+        <v>2957</v>
+      </c>
+      <c r="O480" s="1" t="s">
+        <v>679</v>
+      </c>
+      <c r="U480" s="1" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="478" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B478" s="9" t="s">
-        <v>712</v>
-      </c>
-      <c r="C478" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H478" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="K478" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="L478" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="S478" s="1" t="s">
-        <v>714</v>
-      </c>
-      <c r="U478" s="1" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="479" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B479" s="9" t="s">
-        <v>715</v>
-      </c>
-      <c r="C479" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K479" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="L479" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="S479" s="1" t="s">
-        <v>716</v>
-      </c>
-      <c r="U479" s="1" t="n">
-        <v>3</v>
-      </c>
-    </row>
     <row r="481" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A481" s="1" t="s">
+      <c r="B481" s="1" t="s">
         <v>717</v>
-      </c>
-      <c r="B481" s="1" t="s">
-        <v>718</v>
       </c>
       <c r="C481" s="1" t="s">
         <v>18</v>
@@ -12952,106 +13012,87 @@
       <c r="E481" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F481" s="1" t="n">
-        <v>29</v>
-      </c>
-      <c r="G481" s="1" t="n">
-        <v>2959</v>
-      </c>
-      <c r="H481" s="1" t="s">
-        <v>719</v>
-      </c>
-      <c r="I481" s="1" t="s">
-        <v>720</v>
-      </c>
-      <c r="J481" s="1" t="n">
-        <v>2909</v>
-      </c>
+      <c r="J481" s="1"/>
       <c r="K481" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L481" s="1" t="n">
-        <v>52</v>
-      </c>
-      <c r="N481" s="1" t="n">
-        <v>2957</v>
-      </c>
-      <c r="O481" s="1" t="s">
-        <v>680</v>
+        <v>6</v>
       </c>
       <c r="U481" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="482" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B482" s="1" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
       <c r="C482" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E482" s="1" t="s">
-        <v>19</v>
-      </c>
+      <c r="J482" s="1"/>
       <c r="K482" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L482" s="1" t="n">
         <v>6</v>
       </c>
       <c r="U482" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="483" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B483" s="1" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="C483" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="D483" s="1" t="n">
+        <v>255</v>
+      </c>
+      <c r="J483" s="1"/>
       <c r="K483" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="L483" s="1" t="n">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="S483" s="1" t="s">
+        <v>720</v>
       </c>
       <c r="U483" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="484" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B484" s="1" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="C484" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D484" s="1" t="n">
-        <v>255</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="J484" s="1"/>
       <c r="K484" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="S484" s="1" t="s">
-        <v>724</v>
+        <v>5</v>
+      </c>
+      <c r="L484" s="1" t="n">
+        <v>91</v>
       </c>
       <c r="U484" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="485" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B485" s="1" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="C485" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J485" s="1"/>
       <c r="K485" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L485" s="1" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="U485" s="1" t="n">
         <v>0</v>
@@ -13059,87 +13100,91 @@
     </row>
     <row r="486" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B486" s="1" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="C486" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="H486" s="1" t="s">
+        <v>724</v>
+      </c>
+      <c r="J486" s="1"/>
       <c r="K486" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L486" s="1" t="n">
-        <v>92</v>
+        <v>3</v>
+      </c>
+      <c r="S486" s="1" t="s">
+        <v>725</v>
       </c>
       <c r="U486" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="487" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B487" s="1" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="C487" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H487" s="1" t="s">
-        <v>728</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="J487" s="1"/>
       <c r="K487" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="L487" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="S487" s="1" t="s">
-        <v>729</v>
+        <v>8</v>
       </c>
       <c r="U487" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="488" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B488" s="1" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
       <c r="C488" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D488" s="1" t="n">
-        <v>255</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="J488" s="1"/>
       <c r="K488" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="L488" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="M488" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="S488" s="1" t="s">
+        <v>728</v>
+      </c>
+      <c r="U488" s="1" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="489" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B489" s="9" t="s">
+        <v>729</v>
+      </c>
+      <c r="C489" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J489" s="1"/>
+      <c r="K489" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="L489" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="U488" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="489" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B489" s="1" t="s">
-        <v>731</v>
-      </c>
-      <c r="C489" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K489" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="L489" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="S489" s="1" t="s">
-        <v>732</v>
-      </c>
-      <c r="U489" s="1" t="n">
-        <v>4</v>
-      </c>
+    </row>
+    <row r="490" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="J490" s="1"/>
     </row>
     <row r="491" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A491" s="1" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="B491" s="1" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="C491" s="1" t="s">
         <v>18</v>
@@ -13154,14 +13199,9 @@
         <v>2960</v>
       </c>
       <c r="H491" s="1" t="s">
-        <v>735</v>
-      </c>
-      <c r="I491" s="1" t="s">
-        <v>736</v>
-      </c>
-      <c r="J491" s="1" t="n">
-        <v>2909</v>
-      </c>
+        <v>732</v>
+      </c>
+      <c r="J491" s="1"/>
       <c r="K491" s="1" t="n">
         <v>1</v>
       </c>
@@ -13172,7 +13212,7 @@
         <v>2957</v>
       </c>
       <c r="O491" s="1" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="U491" s="1" t="n">
         <v>0</v>
@@ -13180,7 +13220,7 @@
     </row>
     <row r="492" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B492" s="1" t="s">
-        <v>737</v>
+        <v>733</v>
       </c>
       <c r="C492" s="1" t="s">
         <v>18</v>
@@ -13188,6 +13228,7 @@
       <c r="E492" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="J492" s="1"/>
       <c r="K492" s="1" t="n">
         <v>2</v>
       </c>
@@ -13200,11 +13241,12 @@
     </row>
     <row r="493" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B493" s="1" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
       <c r="C493" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J493" s="1"/>
       <c r="K493" s="1" t="n">
         <v>3</v>
       </c>
@@ -13217,11 +13259,12 @@
     </row>
     <row r="494" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B494" s="1" t="s">
-        <v>739</v>
+        <v>735</v>
       </c>
       <c r="C494" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J494" s="1"/>
       <c r="K494" s="1" t="n">
         <v>4</v>
       </c>
@@ -13229,7 +13272,7 @@
         <v>7</v>
       </c>
       <c r="S494" s="1" t="s">
-        <v>740</v>
+        <v>736</v>
       </c>
       <c r="U494" s="1" t="n">
         <v>3</v>
@@ -13237,11 +13280,12 @@
     </row>
     <row r="495" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B495" s="1" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="C495" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J495" s="1"/>
       <c r="K495" s="1" t="n">
         <v>5</v>
       </c>
@@ -13249,7 +13293,7 @@
         <v>7</v>
       </c>
       <c r="S495" s="1" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="U495" s="1" t="n">
         <v>4</v>
@@ -13257,16 +13301,17 @@
     </row>
     <row r="496" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B496" s="1" t="s">
-        <v>743</v>
+        <v>739</v>
       </c>
       <c r="C496" s="1" t="s">
         <v>113</v>
       </c>
+      <c r="J496" s="1"/>
       <c r="K496" s="1" t="n">
         <v>6</v>
       </c>
       <c r="S496" s="1" t="s">
-        <v>744</v>
+        <v>740</v>
       </c>
       <c r="U496" s="1" t="n">
         <v>2</v>
@@ -13274,68 +13319,49 @@
     </row>
     <row r="497" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B497" s="1" t="s">
-        <v>745</v>
+        <v>741</v>
       </c>
       <c r="C497" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J497" s="1"/>
       <c r="K497" s="1" t="n">
         <v>7</v>
       </c>
       <c r="L497" s="1" t="n">
         <v>7</v>
       </c>
+      <c r="M497" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="U497" s="1" t="n">
         <v>0</v>
       </c>
     </row>
+    <row r="498" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B498" s="9" t="s">
+        <v>742</v>
+      </c>
+      <c r="C498" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J498" s="1"/>
+      <c r="K498" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L498" s="1" t="n">
+        <v>8</v>
+      </c>
+    </row>
     <row r="499" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A499" s="1" t="s">
-        <v>746</v>
-      </c>
-      <c r="B499" s="1" t="s">
-        <v>747</v>
-      </c>
-      <c r="C499" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E499" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F499" s="1" t="n">
-        <v>29</v>
-      </c>
-      <c r="G499" s="1" t="n">
-        <v>2961</v>
-      </c>
-      <c r="H499" s="1" t="s">
-        <v>748</v>
-      </c>
-      <c r="I499" s="1" t="s">
-        <v>749</v>
-      </c>
-      <c r="J499" s="1" t="n">
-        <v>2909</v>
-      </c>
-      <c r="K499" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="L499" s="1" t="n">
-        <v>52</v>
-      </c>
-      <c r="N499" s="1" t="n">
-        <v>2957</v>
-      </c>
-      <c r="O499" s="1" t="s">
-        <v>680</v>
-      </c>
-      <c r="U499" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="J499" s="1"/>
     </row>
     <row r="500" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A500" s="1" t="s">
+        <v>743</v>
+      </c>
       <c r="B500" s="1" t="s">
-        <v>750</v>
+        <v>744</v>
       </c>
       <c r="C500" s="1" t="s">
         <v>18</v>
@@ -13343,42 +13369,66 @@
       <c r="E500" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="F500" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="G500" s="1" t="n">
+        <v>2961</v>
+      </c>
+      <c r="H500" s="1" t="s">
+        <v>745</v>
+      </c>
+      <c r="J500" s="1"/>
       <c r="K500" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L500" s="1" t="n">
-        <v>6</v>
+        <v>52</v>
+      </c>
+      <c r="N500" s="1" t="n">
+        <v>2957</v>
+      </c>
+      <c r="O500" s="1" t="s">
+        <v>679</v>
       </c>
       <c r="U500" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="501" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B501" s="1" t="s">
-        <v>751</v>
+        <v>746</v>
       </c>
       <c r="C501" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="E501" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J501" s="1"/>
       <c r="K501" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L501" s="1" t="n">
         <v>6</v>
       </c>
       <c r="U501" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="502" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B502" s="1" t="s">
-        <v>752</v>
+        <v>747</v>
       </c>
       <c r="C502" s="1" t="s">
-        <v>113</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="J502" s="1"/>
       <c r="K502" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="L502" s="1" t="n">
+        <v>6</v>
       </c>
       <c r="U502" s="1" t="n">
         <v>0</v>
@@ -13386,114 +13436,97 @@
     </row>
     <row r="503" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B503" s="1" t="s">
-        <v>753</v>
+        <v>748</v>
       </c>
       <c r="C503" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H503" s="1" t="s">
-        <v>754</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="J503" s="1"/>
       <c r="K503" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="L503" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="S503" s="1" t="s">
-        <v>755</v>
+        <v>4</v>
       </c>
       <c r="U503" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="504" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B504" s="1" t="s">
-        <v>756</v>
+        <v>749</v>
       </c>
       <c r="C504" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="H504" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="J504" s="1"/>
       <c r="K504" s="1" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L504" s="1" t="n">
         <v>3</v>
       </c>
       <c r="S504" s="1" t="s">
-        <v>757</v>
+        <v>751</v>
       </c>
       <c r="U504" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="505" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B505" s="1" t="s">
-        <v>758</v>
+        <v>752</v>
       </c>
       <c r="C505" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J505" s="1"/>
       <c r="K505" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="L505" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="S505" s="1" t="s">
+        <v>753</v>
+      </c>
+      <c r="U505" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="506" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B506" s="1" t="s">
+        <v>754</v>
+      </c>
+      <c r="C506" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J506" s="1"/>
+      <c r="K506" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="L505" s="1" t="n">
+      <c r="L506" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="S505" s="1" t="s">
-        <v>716</v>
-      </c>
-      <c r="U505" s="1" t="n">
+      <c r="M506" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="S506" s="1" t="s">
+        <v>713</v>
+      </c>
+      <c r="U506" s="1" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="507" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A507" s="1" t="s">
-        <v>759</v>
-      </c>
-      <c r="B507" s="1" t="s">
-        <v>760</v>
-      </c>
-      <c r="C507" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E507" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F507" s="1" t="n">
-        <v>29</v>
-      </c>
-      <c r="G507" s="1" t="n">
-        <v>2962</v>
-      </c>
-      <c r="H507" s="1" t="s">
-        <v>761</v>
-      </c>
-      <c r="I507" s="1" t="s">
-        <v>762</v>
-      </c>
-      <c r="J507" s="1" t="n">
-        <v>2909</v>
-      </c>
-      <c r="K507" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="L507" s="1" t="n">
-        <v>52</v>
-      </c>
-      <c r="N507" s="1" t="n">
-        <v>2957</v>
-      </c>
-      <c r="O507" s="1" t="s">
-        <v>680</v>
-      </c>
-      <c r="U507" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="J507" s="1"/>
     </row>
     <row r="508" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A508" s="1" t="s">
+        <v>755</v>
+      </c>
       <c r="B508" s="1" t="s">
-        <v>763</v>
+        <v>756</v>
       </c>
       <c r="C508" s="1" t="s">
         <v>18</v>
@@ -13501,142 +13534,195 @@
       <c r="E508" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="F508" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="G508" s="1" t="n">
+        <v>2962</v>
+      </c>
+      <c r="H508" s="1" t="s">
+        <v>757</v>
+      </c>
+      <c r="J508" s="1"/>
       <c r="K508" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L508" s="1" t="n">
-        <v>6</v>
+        <v>52</v>
+      </c>
+      <c r="N508" s="1" t="n">
+        <v>2957</v>
+      </c>
+      <c r="O508" s="1" t="s">
+        <v>679</v>
       </c>
       <c r="U508" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="509" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B509" s="1" t="s">
-        <v>764</v>
+        <v>758</v>
       </c>
       <c r="C509" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="E509" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J509" s="1"/>
       <c r="K509" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L509" s="1" t="n">
         <v>6</v>
       </c>
       <c r="U509" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="510" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B510" s="1" t="s">
-        <v>765</v>
+        <v>759</v>
       </c>
       <c r="C510" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J510" s="1"/>
+      <c r="K510" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L510" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="U510" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="511" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B511" s="1" t="s">
+        <v>760</v>
+      </c>
+      <c r="C511" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="K510" s="1" t="n">
+      <c r="J511" s="1"/>
+      <c r="K511" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="S510" s="1" t="s">
+      <c r="S511" s="1" t="s">
         <v>594</v>
       </c>
-      <c r="U510" s="1" t="n">
+      <c r="U511" s="1" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="511" customFormat="false" ht="15" hidden="true" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="512" customFormat="false" ht="15" hidden="true" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="512" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B512" s="1" t="s">
+        <v>761</v>
+      </c>
+      <c r="C512" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J512" s="1"/>
+      <c r="K512" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="L512" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="S512" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="U512" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
     <row r="513" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B513" s="1" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="C513" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J513" s="1"/>
       <c r="K513" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L513" s="1" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S513" s="1" t="s">
-        <v>650</v>
+        <v>763</v>
       </c>
       <c r="U513" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="514" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B514" s="1" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
       <c r="C514" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="H514" s="1" t="s">
+        <v>765</v>
+      </c>
+      <c r="J514" s="1"/>
       <c r="K514" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L514" s="1" t="n">
-        <v>7</v>
+        <v>31</v>
+      </c>
+      <c r="N514" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="O514" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="P514" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="Q514" s="1" t="s">
+        <v>501</v>
       </c>
       <c r="S514" s="1" t="s">
-        <v>768</v>
+        <v>502</v>
       </c>
       <c r="U514" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="515" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B515" s="1" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
       <c r="C515" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H515" s="1" t="s">
-        <v>770</v>
-      </c>
+      <c r="J515" s="1"/>
       <c r="K515" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L515" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="L515" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="M515" s="1" t="n">
-        <v>31</v>
-      </c>
-      <c r="N515" s="1" t="s">
-        <v>498</v>
-      </c>
-      <c r="O515" s="1" t="s">
-        <v>499</v>
-      </c>
-      <c r="P515" s="1" t="s">
-        <v>500</v>
-      </c>
-      <c r="Q515" s="1" t="s">
-        <v>501</v>
-      </c>
-      <c r="S515" s="1" t="s">
-        <v>502</v>
-      </c>
       <c r="U515" s="1" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="516" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B516" s="1" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="C516" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="J516" s="1"/>
       <c r="K516" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="L516" s="1" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="U516" s="1" t="n">
         <v>0</v>
@@ -13644,41 +13730,70 @@
     </row>
     <row r="517" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B517" s="1" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="C517" s="1" t="s">
-        <v>113</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="J517" s="1"/>
       <c r="K517" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="L517" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="M517" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="U517" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="518" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B518" s="1" t="s">
-        <v>773</v>
-      </c>
-      <c r="C518" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K518" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="L518" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="U518" s="1" t="n">
+      <c r="J518" s="1"/>
+    </row>
+    <row r="519" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A519" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="B519" s="1" t="s">
+        <v>770</v>
+      </c>
+      <c r="C519" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E519" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F519" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="G519" s="1" t="n">
+        <v>2963</v>
+      </c>
+      <c r="H519" s="1" t="s">
+        <v>771</v>
+      </c>
+      <c r="J519" s="1"/>
+      <c r="K519" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L519" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="N519" s="1" t="n">
+        <v>2957</v>
+      </c>
+      <c r="O519" s="1" t="s">
+        <v>679</v>
+      </c>
+      <c r="U519" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="520" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A520" s="1" t="s">
-        <v>774</v>
-      </c>
       <c r="B520" s="1" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
       <c r="C520" s="1" t="s">
         <v>18</v>
@@ -13686,69 +13801,45 @@
       <c r="E520" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F520" s="1" t="n">
-        <v>29</v>
-      </c>
-      <c r="G520" s="1" t="n">
-        <v>2963</v>
-      </c>
-      <c r="H520" s="1" t="s">
-        <v>776</v>
-      </c>
-      <c r="I520" s="1" t="s">
-        <v>777</v>
-      </c>
-      <c r="J520" s="1" t="n">
-        <v>2909</v>
-      </c>
+      <c r="J520" s="1"/>
       <c r="K520" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L520" s="1" t="n">
-        <v>52</v>
-      </c>
-      <c r="N520" s="1" t="n">
-        <v>2957</v>
-      </c>
-      <c r="O520" s="1" t="s">
-        <v>680</v>
+        <v>6</v>
       </c>
       <c r="U520" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="521" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B521" s="1" t="s">
-        <v>778</v>
+        <v>773</v>
       </c>
       <c r="C521" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E521" s="1" t="s">
-        <v>19</v>
-      </c>
+      <c r="J521" s="1"/>
       <c r="K521" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L521" s="1" t="n">
         <v>6</v>
       </c>
       <c r="U521" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="522" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B522" s="1" t="s">
-        <v>779</v>
+        <v>774</v>
       </c>
       <c r="C522" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="J522" s="1"/>
       <c r="K522" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="L522" s="1" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U522" s="1" t="n">
         <v>0</v>
@@ -13756,147 +13847,218 @@
     </row>
     <row r="523" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B523" s="1" t="s">
-        <v>780</v>
+        <v>775</v>
       </c>
       <c r="C523" s="1" t="s">
-        <v>113</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="J523" s="1"/>
       <c r="K523" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="L523" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="S523" s="1" t="s">
+        <v>776</v>
       </c>
       <c r="U523" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="524" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B524" s="1" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="C524" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D524" s="1" t="n">
-        <v>100</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="H524" s="1" t="s">
+        <v>778</v>
+      </c>
+      <c r="J524" s="1"/>
       <c r="K524" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="L524" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="N524" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="O524" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="P524" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="Q524" s="1" t="s">
+        <v>501</v>
       </c>
       <c r="S524" s="1" t="s">
-        <v>782</v>
+        <v>502</v>
       </c>
       <c r="U524" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="525" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B525" s="1" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="C525" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J525" s="1"/>
       <c r="K525" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L525" s="1" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S525" s="1" t="s">
-        <v>784</v>
+        <v>780</v>
       </c>
       <c r="U525" s="1" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="526" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B526" s="1" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="C526" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H526" s="1" t="s">
-        <v>786</v>
-      </c>
+      <c r="J526" s="1"/>
       <c r="K526" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L526" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="L526" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="M526" s="1" t="n">
-        <v>31</v>
-      </c>
-      <c r="N526" s="1" t="s">
-        <v>498</v>
-      </c>
-      <c r="O526" s="1" t="s">
-        <v>499</v>
-      </c>
-      <c r="P526" s="1" t="s">
-        <v>500</v>
-      </c>
-      <c r="Q526" s="1" t="s">
-        <v>501</v>
-      </c>
-      <c r="S526" s="1" t="s">
-        <v>502</v>
-      </c>
       <c r="U526" s="1" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="527" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B527" s="1" t="s">
-        <v>787</v>
+        <v>782</v>
       </c>
       <c r="C527" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="J527" s="1"/>
       <c r="K527" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="L527" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="S527" s="1" t="s">
-        <v>788</v>
+        <v>9</v>
       </c>
       <c r="U527" s="1" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="528" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B528" s="1" t="s">
-        <v>789</v>
-      </c>
-      <c r="C528" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K528" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="L528" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="U528" s="1" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="529" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B529" s="1" t="s">
-        <v>790</v>
-      </c>
-      <c r="C529" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="K529" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="U529" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    <row r="1048469" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048470" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048471" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048472" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048473" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048474" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048475" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048476" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048477" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048478" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048479" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048480" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048481" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048482" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048483" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048484" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048485" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048486" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048487" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048488" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048489" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048490" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048491" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048492" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048493" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048494" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048495" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048496" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048497" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048498" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048499" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048500" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048501" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048502" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048503" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048504" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048505" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048506" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048507" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048508" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048509" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048510" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048511" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048512" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048513" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048514" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048515" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048516" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048517" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048518" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048519" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048520" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048521" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048522" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048523" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048524" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048525" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048526" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048527" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048528" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048529" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048530" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048531" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048532" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048533" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048534" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048535" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048536" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048537" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048538" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048539" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048540" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048541" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048542" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048543" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048544" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048545" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048546" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048547" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048548" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048549" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048550" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048551" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048552" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>